<commit_message>
status save button added
</commit_message>
<xml_diff>
--- a/storage/app/Colombo_status_upload.xlsx
+++ b/storage/app/Colombo_status_upload.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
   <si>
     <t>Handle By</t>
   </si>
@@ -48,6 +48,18 @@
   </si>
   <si>
     <t>2025/10/31</t>
+  </si>
+  <si>
+    <t>Sri Lanka</t>
+  </si>
+  <si>
+    <t>2025/05/08</t>
+  </si>
+  <si>
+    <t>001</t>
+  </si>
+  <si>
+    <t>accept</t>
   </si>
 </sst>
 </file>
@@ -434,13 +446,27 @@
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2">
+        <v>10</v>
+      </c>
+      <c r="H2">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>14</v>
+      </c>
       <c r="J2"/>
       <c r="K2"/>
       <c r="L2"/>

</xml_diff>